<commit_message>
Apply relabels: Timeline for new feature -> CONSULT(Meta: Migration/Timeline Question); Request to deactivate template -> CONSULT(Information: How To / Procedure). Regenerate statistics files (consolidated + detailed).
</commit_message>
<xml_diff>
--- a/Statistics_Latest_Consolidated.xlsx
+++ b/Statistics_Latest_Consolidated.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,15 +30,9 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -49,18 +43,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
         <bgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0070AD47"/>
-        <bgColor rgb="0070AD47"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,14 +58,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -449,19 +428,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -486,27 +454,27 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Median_Hours</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Min_Hours</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Max_Hours</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Avg_Days</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Median_Hours</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Median_Days</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Min_Hours</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Max_Hours</t>
         </is>
       </c>
     </row>
@@ -520,25 +488,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D2" t="n">
-        <v>233.34</v>
+        <v>237.78</v>
       </c>
       <c r="E2" t="n">
-        <v>9.720000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>96.75</v>
+        <v>0.18</v>
       </c>
       <c r="G2" t="n">
-        <v>4.03</v>
+        <v>2748.68</v>
       </c>
       <c r="H2" t="n">
-        <v>0.18</v>
+        <v>9.91</v>
       </c>
       <c r="I2" t="n">
-        <v>2748.68</v>
+        <v>4.04</v>
       </c>
     </row>
     <row r="3">
@@ -557,19 +525,19 @@
         <v>762.37</v>
       </c>
       <c r="E3" t="n">
+        <v>530.13</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3089.68</v>
+      </c>
+      <c r="H3" t="n">
         <v>31.77</v>
       </c>
-      <c r="F3" t="n">
-        <v>530.13</v>
-      </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>22.09</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2.32</v>
-      </c>
-      <c r="I3" t="n">
-        <v>3089.68</v>
       </c>
     </row>
     <row r="4">
@@ -588,19 +556,19 @@
         <v>327.87</v>
       </c>
       <c r="E4" t="n">
+        <v>176.59</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2535.75</v>
+      </c>
+      <c r="H4" t="n">
         <v>13.66</v>
       </c>
-      <c r="F4" t="n">
-        <v>176.59</v>
-      </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>7.36</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="I4" t="n">
-        <v>2535.75</v>
       </c>
     </row>
     <row r="5">
@@ -619,19 +587,19 @@
         <v>165.68</v>
       </c>
       <c r="E5" t="n">
+        <v>61.48</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1224.93</v>
+      </c>
+      <c r="H5" t="n">
         <v>6.9</v>
       </c>
-      <c r="F5" t="n">
-        <v>61.48</v>
-      </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>2.56</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1224.93</v>
       </c>
     </row>
     <row r="6">
@@ -650,19 +618,19 @@
         <v>245.21</v>
       </c>
       <c r="E6" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3747.8</v>
+      </c>
+      <c r="H6" t="n">
         <v>10.22</v>
       </c>
-      <c r="F6" t="n">
-        <v>26.9</v>
-      </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>1.12</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="I6" t="n">
-        <v>3747.8</v>
       </c>
     </row>
     <row r="7">
@@ -681,19 +649,19 @@
         <v>133.27</v>
       </c>
       <c r="E7" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1234.32</v>
+      </c>
+      <c r="H7" t="n">
         <v>5.55</v>
       </c>
-      <c r="F7" t="n">
-        <v>23.4</v>
-      </c>
-      <c r="G7" t="n">
+      <c r="I7" t="n">
         <v>0.98</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="I7" t="n">
-        <v>1234.32</v>
       </c>
     </row>
     <row r="8">
@@ -712,19 +680,19 @@
         <v>193.42</v>
       </c>
       <c r="E8" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1275.23</v>
+      </c>
+      <c r="H8" t="n">
         <v>8.06</v>
       </c>
-      <c r="F8" t="n">
-        <v>96.8</v>
-      </c>
-      <c r="G8" t="n">
+      <c r="I8" t="n">
         <v>4.03</v>
-      </c>
-      <c r="H8" t="n">
-        <v>2.23</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1275.23</v>
       </c>
     </row>
     <row r="9">
@@ -743,19 +711,19 @@
         <v>324.7</v>
       </c>
       <c r="E9" t="n">
+        <v>200.12</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1387.98</v>
+      </c>
+      <c r="H9" t="n">
         <v>13.53</v>
       </c>
-      <c r="F9" t="n">
-        <v>200.12</v>
-      </c>
-      <c r="G9" t="n">
+      <c r="I9" t="n">
         <v>8.34</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="I9" t="n">
-        <v>1387.98</v>
       </c>
     </row>
     <row r="10">
@@ -764,29 +732,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Archiving</t>
+          <t>Request account for user</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>29</v>
       </c>
       <c r="D10" t="n">
-        <v>118.48</v>
+        <v>36.14</v>
       </c>
       <c r="E10" t="n">
-        <v>4.94</v>
+        <v>17.03</v>
       </c>
       <c r="F10" t="n">
-        <v>26.87</v>
+        <v>1.22</v>
       </c>
       <c r="G10" t="n">
-        <v>1.12</v>
+        <v>145.72</v>
       </c>
       <c r="H10" t="n">
-        <v>2.22</v>
+        <v>1.51</v>
       </c>
       <c r="I10" t="n">
-        <v>881.92</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="11">
@@ -795,29 +763,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Request account for user</t>
+          <t>Archiving</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>29</v>
       </c>
       <c r="D11" t="n">
-        <v>36.14</v>
+        <v>118.48</v>
       </c>
       <c r="E11" t="n">
-        <v>1.51</v>
+        <v>26.87</v>
       </c>
       <c r="F11" t="n">
-        <v>17.03</v>
+        <v>2.22</v>
       </c>
       <c r="G11" t="n">
-        <v>0.71</v>
+        <v>881.92</v>
       </c>
       <c r="H11" t="n">
-        <v>1.22</v>
+        <v>4.94</v>
       </c>
       <c r="I11" t="n">
-        <v>145.72</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="12">
@@ -826,29 +794,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Forward the request to new approver</t>
+          <t>Attachment Issue</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>18</v>
       </c>
       <c r="D12" t="n">
-        <v>89.88</v>
+        <v>253.92</v>
       </c>
       <c r="E12" t="n">
-        <v>3.74</v>
+        <v>186.54</v>
       </c>
       <c r="F12" t="n">
-        <v>25.45</v>
+        <v>0.05</v>
       </c>
       <c r="G12" t="n">
-        <v>1.06</v>
+        <v>977.48</v>
       </c>
       <c r="H12" t="n">
-        <v>0.33</v>
+        <v>10.58</v>
       </c>
       <c r="I12" t="n">
-        <v>356.45</v>
+        <v>7.77</v>
       </c>
     </row>
     <row r="13">
@@ -857,29 +825,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Attachment Issue</t>
+          <t>Forward the request to new approver</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>18</v>
       </c>
       <c r="D13" t="n">
-        <v>253.92</v>
+        <v>89.88</v>
       </c>
       <c r="E13" t="n">
-        <v>10.58</v>
+        <v>25.45</v>
       </c>
       <c r="F13" t="n">
-        <v>186.54</v>
+        <v>0.33</v>
       </c>
       <c r="G13" t="n">
-        <v>7.77</v>
+        <v>356.45</v>
       </c>
       <c r="H13" t="n">
-        <v>0.05</v>
+        <v>3.74</v>
       </c>
       <c r="I13" t="n">
-        <v>977.48</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="14">
@@ -898,19 +866,19 @@
         <v>372.22</v>
       </c>
       <c r="E14" t="n">
+        <v>241.87</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6.28</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2160.17</v>
+      </c>
+      <c r="H14" t="n">
         <v>15.51</v>
       </c>
-      <c r="F14" t="n">
-        <v>241.87</v>
-      </c>
-      <c r="G14" t="n">
+      <c r="I14" t="n">
         <v>10.08</v>
-      </c>
-      <c r="H14" t="n">
-        <v>6.28</v>
-      </c>
-      <c r="I14" t="n">
-        <v>2160.17</v>
       </c>
     </row>
     <row r="15">
@@ -929,19 +897,19 @@
         <v>124.83</v>
       </c>
       <c r="E15" t="n">
+        <v>57.64</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G15" t="n">
+        <v>479.92</v>
+      </c>
+      <c r="H15" t="n">
         <v>5.2</v>
       </c>
-      <c r="F15" t="n">
-        <v>57.64</v>
-      </c>
-      <c r="G15" t="n">
+      <c r="I15" t="n">
         <v>2.4</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="I15" t="n">
-        <v>479.92</v>
       </c>
     </row>
     <row r="16">
@@ -960,19 +928,19 @@
         <v>160.02</v>
       </c>
       <c r="E16" t="n">
+        <v>95.75</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G16" t="n">
+        <v>528.22</v>
+      </c>
+      <c r="H16" t="n">
         <v>6.67</v>
       </c>
-      <c r="F16" t="n">
-        <v>95.75</v>
-      </c>
-      <c r="G16" t="n">
+      <c r="I16" t="n">
         <v>3.99</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="I16" t="n">
-        <v>528.22</v>
       </c>
     </row>
     <row r="17">
@@ -991,19 +959,19 @@
         <v>177.93</v>
       </c>
       <c r="E17" t="n">
+        <v>154.18</v>
+      </c>
+      <c r="F17" t="n">
+        <v>69.05</v>
+      </c>
+      <c r="G17" t="n">
+        <v>502.6</v>
+      </c>
+      <c r="H17" t="n">
         <v>7.41</v>
       </c>
-      <c r="F17" t="n">
-        <v>154.18</v>
-      </c>
-      <c r="G17" t="n">
+      <c r="I17" t="n">
         <v>6.42</v>
-      </c>
-      <c r="H17" t="n">
-        <v>69.05</v>
-      </c>
-      <c r="I17" t="n">
-        <v>502.6</v>
       </c>
     </row>
     <row r="18">
@@ -1022,19 +990,19 @@
         <v>54.34</v>
       </c>
       <c r="E18" t="n">
+        <v>24.43</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="G18" t="n">
+        <v>166.98</v>
+      </c>
+      <c r="H18" t="n">
         <v>2.26</v>
       </c>
-      <c r="F18" t="n">
-        <v>24.43</v>
-      </c>
-      <c r="G18" t="n">
+      <c r="I18" t="n">
         <v>1.02</v>
-      </c>
-      <c r="H18" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="I18" t="n">
-        <v>166.98</v>
       </c>
     </row>
     <row r="19">
@@ -1053,19 +1021,19 @@
         <v>345.24</v>
       </c>
       <c r="E19" t="n">
+        <v>406.28</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="G19" t="n">
+        <v>679.05</v>
+      </c>
+      <c r="H19" t="n">
         <v>14.38</v>
       </c>
-      <c r="F19" t="n">
-        <v>406.28</v>
-      </c>
-      <c r="G19" t="n">
+      <c r="I19" t="n">
         <v>16.93</v>
-      </c>
-      <c r="H19" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="I19" t="n">
-        <v>679.05</v>
       </c>
     </row>
     <row r="20">
@@ -1084,19 +1052,19 @@
         <v>841.16</v>
       </c>
       <c r="E20" t="n">
+        <v>603.25</v>
+      </c>
+      <c r="F20" t="n">
+        <v>120.9</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2019.82</v>
+      </c>
+      <c r="H20" t="n">
         <v>35.05</v>
       </c>
-      <c r="F20" t="n">
-        <v>603.25</v>
-      </c>
-      <c r="G20" t="n">
+      <c r="I20" t="n">
         <v>25.14</v>
-      </c>
-      <c r="H20" t="n">
-        <v>120.9</v>
-      </c>
-      <c r="I20" t="n">
-        <v>2019.82</v>
       </c>
     </row>
     <row r="21">
@@ -1115,19 +1083,19 @@
         <v>217.17</v>
       </c>
       <c r="E21" t="n">
+        <v>242.8</v>
+      </c>
+      <c r="F21" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="G21" t="n">
+        <v>535.22</v>
+      </c>
+      <c r="H21" t="n">
         <v>9.050000000000001</v>
       </c>
-      <c r="F21" t="n">
-        <v>242.8</v>
-      </c>
-      <c r="G21" t="n">
+      <c r="I21" t="n">
         <v>10.12</v>
-      </c>
-      <c r="H21" t="n">
-        <v>6.63</v>
-      </c>
-      <c r="I21" t="n">
-        <v>535.22</v>
       </c>
     </row>
     <row r="22">
@@ -1146,19 +1114,19 @@
         <v>59.34</v>
       </c>
       <c r="E22" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G22" t="n">
+        <v>304.37</v>
+      </c>
+      <c r="H22" t="n">
         <v>2.47</v>
       </c>
-      <c r="F22" t="n">
-        <v>8.77</v>
-      </c>
-      <c r="G22" t="n">
+      <c r="I22" t="n">
         <v>0.37</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I22" t="n">
-        <v>304.37</v>
       </c>
     </row>
     <row r="23">
@@ -1177,19 +1145,19 @@
         <v>307.38</v>
       </c>
       <c r="E23" t="n">
+        <v>211.5</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="G23" t="n">
+        <v>926.7</v>
+      </c>
+      <c r="H23" t="n">
         <v>12.81</v>
       </c>
-      <c r="F23" t="n">
-        <v>211.5</v>
-      </c>
-      <c r="G23" t="n">
+      <c r="I23" t="n">
         <v>8.81</v>
-      </c>
-      <c r="H23" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="I23" t="n">
-        <v>926.7</v>
       </c>
     </row>
     <row r="24">
@@ -1208,19 +1176,19 @@
         <v>597.73</v>
       </c>
       <c r="E24" t="n">
+        <v>282.78</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1517.08</v>
+      </c>
+      <c r="H24" t="n">
         <v>24.91</v>
       </c>
-      <c r="F24" t="n">
-        <v>282.78</v>
-      </c>
-      <c r="G24" t="n">
+      <c r="I24" t="n">
         <v>11.78</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="I24" t="n">
-        <v>1517.08</v>
       </c>
     </row>
     <row r="25">
@@ -1239,19 +1207,19 @@
         <v>1238.26</v>
       </c>
       <c r="E25" t="n">
+        <v>551.66</v>
+      </c>
+      <c r="F25" t="n">
+        <v>116</v>
+      </c>
+      <c r="G25" t="n">
+        <v>3716.62</v>
+      </c>
+      <c r="H25" t="n">
         <v>51.59</v>
       </c>
-      <c r="F25" t="n">
-        <v>551.66</v>
-      </c>
-      <c r="G25" t="n">
+      <c r="I25" t="n">
         <v>22.99</v>
-      </c>
-      <c r="H25" t="n">
-        <v>116</v>
-      </c>
-      <c r="I25" t="n">
-        <v>3716.62</v>
       </c>
     </row>
     <row r="26">
@@ -1270,19 +1238,19 @@
         <v>160.2</v>
       </c>
       <c r="E26" t="n">
+        <v>25.89</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="G26" t="n">
+        <v>541.97</v>
+      </c>
+      <c r="H26" t="n">
         <v>6.68</v>
       </c>
-      <c r="F26" t="n">
-        <v>25.89</v>
-      </c>
-      <c r="G26" t="n">
+      <c r="I26" t="n">
         <v>1.08</v>
-      </c>
-      <c r="H26" t="n">
-        <v>2.53</v>
-      </c>
-      <c r="I26" t="n">
-        <v>541.97</v>
       </c>
     </row>
     <row r="27">
@@ -1301,19 +1269,19 @@
         <v>540.26</v>
       </c>
       <c r="E27" t="n">
+        <v>168.92</v>
+      </c>
+      <c r="F27" t="n">
+        <v>15.22</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1457.87</v>
+      </c>
+      <c r="H27" t="n">
         <v>22.51</v>
       </c>
-      <c r="F27" t="n">
-        <v>168.92</v>
-      </c>
-      <c r="G27" t="n">
+      <c r="I27" t="n">
         <v>7.04</v>
-      </c>
-      <c r="H27" t="n">
-        <v>15.22</v>
-      </c>
-      <c r="I27" t="n">
-        <v>1457.87</v>
       </c>
     </row>
     <row r="28">
@@ -1332,19 +1300,19 @@
         <v>314.95</v>
       </c>
       <c r="E28" t="n">
+        <v>302.23</v>
+      </c>
+      <c r="F28" t="n">
+        <v>22.22</v>
+      </c>
+      <c r="G28" t="n">
+        <v>665.52</v>
+      </c>
+      <c r="H28" t="n">
         <v>13.12</v>
       </c>
-      <c r="F28" t="n">
-        <v>302.23</v>
-      </c>
-      <c r="G28" t="n">
+      <c r="I28" t="n">
         <v>12.59</v>
-      </c>
-      <c r="H28" t="n">
-        <v>22.22</v>
-      </c>
-      <c r="I28" t="n">
-        <v>665.52</v>
       </c>
     </row>
     <row r="29">
@@ -1363,19 +1331,19 @@
         <v>241.79</v>
       </c>
       <c r="E29" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G29" t="n">
+        <v>1193.6</v>
+      </c>
+      <c r="H29" t="n">
         <v>10.07</v>
       </c>
-      <c r="F29" t="n">
-        <v>2.37</v>
-      </c>
-      <c r="G29" t="n">
+      <c r="I29" t="n">
         <v>0.1</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="I29" t="n">
-        <v>1193.6</v>
       </c>
     </row>
     <row r="30">
@@ -1394,19 +1362,19 @@
         <v>88.63</v>
       </c>
       <c r="E30" t="n">
+        <v>117.97</v>
+      </c>
+      <c r="F30" t="n">
+        <v>13.62</v>
+      </c>
+      <c r="G30" t="n">
+        <v>134.32</v>
+      </c>
+      <c r="H30" t="n">
         <v>3.69</v>
       </c>
-      <c r="F30" t="n">
-        <v>117.97</v>
-      </c>
-      <c r="G30" t="n">
+      <c r="I30" t="n">
         <v>4.92</v>
-      </c>
-      <c r="H30" t="n">
-        <v>13.62</v>
-      </c>
-      <c r="I30" t="n">
-        <v>134.32</v>
       </c>
     </row>
     <row r="31">
@@ -1425,19 +1393,19 @@
         <v>115.56</v>
       </c>
       <c r="E31" t="n">
+        <v>115.56</v>
+      </c>
+      <c r="F31" t="n">
+        <v>66.81999999999999</v>
+      </c>
+      <c r="G31" t="n">
+        <v>164.3</v>
+      </c>
+      <c r="H31" t="n">
         <v>4.82</v>
       </c>
-      <c r="F31" t="n">
-        <v>115.56</v>
-      </c>
-      <c r="G31" t="n">
+      <c r="I31" t="n">
         <v>4.82</v>
-      </c>
-      <c r="H31" t="n">
-        <v>66.81999999999999</v>
-      </c>
-      <c r="I31" t="n">
-        <v>164.3</v>
       </c>
     </row>
     <row r="32">
@@ -1456,19 +1424,19 @@
         <v>409.54</v>
       </c>
       <c r="E32" t="n">
+        <v>409.54</v>
+      </c>
+      <c r="F32" t="n">
+        <v>164.65</v>
+      </c>
+      <c r="G32" t="n">
+        <v>654.4299999999999</v>
+      </c>
+      <c r="H32" t="n">
         <v>17.06</v>
       </c>
-      <c r="F32" t="n">
-        <v>409.54</v>
-      </c>
-      <c r="G32" t="n">
+      <c r="I32" t="n">
         <v>17.06</v>
-      </c>
-      <c r="H32" t="n">
-        <v>164.65</v>
-      </c>
-      <c r="I32" t="n">
-        <v>654.4299999999999</v>
       </c>
     </row>
     <row r="33">
@@ -1487,19 +1455,19 @@
         <v>62.79</v>
       </c>
       <c r="E33" t="n">
+        <v>62.79</v>
+      </c>
+      <c r="F33" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="G33" t="n">
+        <v>100.73</v>
+      </c>
+      <c r="H33" t="n">
         <v>2.62</v>
       </c>
-      <c r="F33" t="n">
-        <v>62.79</v>
-      </c>
-      <c r="G33" t="n">
+      <c r="I33" t="n">
         <v>2.62</v>
-      </c>
-      <c r="H33" t="n">
-        <v>24.85</v>
-      </c>
-      <c r="I33" t="n">
-        <v>100.73</v>
       </c>
     </row>
     <row r="34">
@@ -1508,91 +1476,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Request to deactivate template</t>
+          <t>UNCLASSIFIED</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>862.87</v>
+        <v>184.77</v>
       </c>
       <c r="E34" t="n">
-        <v>35.95</v>
+        <v>184.77</v>
       </c>
       <c r="F34" t="n">
-        <v>862.87</v>
+        <v>184.77</v>
       </c>
       <c r="G34" t="n">
-        <v>35.95</v>
+        <v>184.77</v>
       </c>
       <c r="H34" t="n">
-        <v>862.87</v>
+        <v>7.7</v>
       </c>
       <c r="I34" t="n">
-        <v>862.87</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Timeline for new feature</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" t="n">
-        <v>1204.42</v>
-      </c>
-      <c r="E35" t="n">
-        <v>50.18</v>
-      </c>
-      <c r="F35" t="n">
-        <v>1204.42</v>
-      </c>
-      <c r="G35" t="n">
-        <v>50.18</v>
-      </c>
-      <c r="H35" t="n">
-        <v>1204.42</v>
-      </c>
-      <c r="I35" t="n">
-        <v>1204.42</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>UNCLASSIFIED</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" t="n">
-        <v>184.77</v>
-      </c>
-      <c r="E36" t="n">
         <v>7.7</v>
-      </c>
-      <c r="F36" t="n">
-        <v>184.77</v>
-      </c>
-      <c r="G36" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="H36" t="n">
-        <v>184.77</v>
-      </c>
-      <c r="I36" t="n">
-        <v>184.77</v>
       </c>
     </row>
   </sheetData>
@@ -1606,16 +1512,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1645,7 +1543,22 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Min_Hours</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Max_Hours</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Avg_Days</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Median_Days</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1583,16 @@
         <v>2.37</v>
       </c>
       <c r="F2" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1193.6</v>
+      </c>
+      <c r="H2" t="n">
         <v>10.07</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="3">
@@ -1694,7 +1616,16 @@
         <v>24.43</v>
       </c>
       <c r="F3" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="G3" t="n">
+        <v>166.98</v>
+      </c>
+      <c r="H3" t="n">
         <v>2.26</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1.02</v>
       </c>
     </row>
     <row r="4">
@@ -1718,7 +1649,16 @@
         <v>26.87</v>
       </c>
       <c r="F4" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="G4" t="n">
+        <v>881.92</v>
+      </c>
+      <c r="H4" t="n">
         <v>4.94</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.12</v>
       </c>
     </row>
     <row r="5">
@@ -1742,7 +1682,16 @@
         <v>557.87</v>
       </c>
       <c r="F5" t="n">
+        <v>184.77</v>
+      </c>
+      <c r="G5" t="n">
+        <v>619.38</v>
+      </c>
+      <c r="H5" t="n">
         <v>18.92</v>
+      </c>
+      <c r="I5" t="n">
+        <v>23.24</v>
       </c>
     </row>
     <row r="6">
@@ -1766,7 +1715,16 @@
         <v>167.88</v>
       </c>
       <c r="F6" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G6" t="n">
+        <v>977.48</v>
+      </c>
+      <c r="H6" t="n">
         <v>8.91</v>
+      </c>
+      <c r="I6" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -1790,7 +1748,16 @@
         <v>117.17</v>
       </c>
       <c r="F7" t="n">
+        <v>22.22</v>
+      </c>
+      <c r="G7" t="n">
+        <v>665.52</v>
+      </c>
+      <c r="H7" t="n">
         <v>11.18</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.88</v>
       </c>
     </row>
     <row r="8">
@@ -1814,7 +1781,16 @@
         <v>313.33</v>
       </c>
       <c r="F8" t="n">
+        <v>291.13</v>
+      </c>
+      <c r="G8" t="n">
+        <v>480.33</v>
+      </c>
+      <c r="H8" t="n">
         <v>15.07</v>
+      </c>
+      <c r="I8" t="n">
+        <v>13.06</v>
       </c>
     </row>
     <row r="9">
@@ -1829,16 +1805,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D9" t="n">
-        <v>165.42</v>
+        <v>180.7</v>
       </c>
       <c r="E9" t="n">
-        <v>74</v>
+        <v>74.37</v>
       </c>
       <c r="F9" t="n">
-        <v>6.89</v>
+        <v>0.18</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1204.42</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7.53</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3.1</v>
       </c>
     </row>
     <row r="10">
@@ -1853,16 +1838,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D10" t="n">
-        <v>248.93</v>
+        <v>251.02</v>
       </c>
       <c r="E10" t="n">
-        <v>99.72</v>
+        <v>100.73</v>
       </c>
       <c r="F10" t="n">
-        <v>10.37</v>
+        <v>0.45</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2748.68</v>
+      </c>
+      <c r="H10" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="11">
@@ -1886,7 +1880,16 @@
         <v>187.47</v>
       </c>
       <c r="F11" t="n">
+        <v>39.47</v>
+      </c>
+      <c r="G11" t="n">
+        <v>580.38</v>
+      </c>
+      <c r="H11" t="n">
         <v>9.6</v>
+      </c>
+      <c r="I11" t="n">
+        <v>7.81</v>
       </c>
     </row>
     <row r="12">
@@ -1910,7 +1913,16 @@
         <v>309.06</v>
       </c>
       <c r="F12" t="n">
+        <v>6.28</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2160.17</v>
+      </c>
+      <c r="H12" t="n">
         <v>19.05</v>
+      </c>
+      <c r="I12" t="n">
+        <v>12.88</v>
       </c>
     </row>
     <row r="13">
@@ -1934,6 +1946,15 @@
         <v>109.32</v>
       </c>
       <c r="F13" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="G13" t="n">
+        <v>211.5</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="I13" t="n">
         <v>4.56</v>
       </c>
     </row>
@@ -1958,7 +1979,16 @@
         <v>359.23</v>
       </c>
       <c r="F14" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="G14" t="n">
+        <v>926.7</v>
+      </c>
+      <c r="H14" t="n">
         <v>16.11</v>
+      </c>
+      <c r="I14" t="n">
+        <v>14.97</v>
       </c>
     </row>
     <row r="15">
@@ -1982,7 +2012,16 @@
         <v>210.68</v>
       </c>
       <c r="F15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1960.83</v>
+      </c>
+      <c r="H15" t="n">
         <v>15.85</v>
+      </c>
+      <c r="I15" t="n">
+        <v>8.779999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -2006,7 +2045,16 @@
         <v>174.57</v>
       </c>
       <c r="F16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2535.75</v>
+      </c>
+      <c r="H16" t="n">
         <v>13.38</v>
+      </c>
+      <c r="I16" t="n">
+        <v>7.27</v>
       </c>
     </row>
     <row r="17">
@@ -2030,7 +2078,16 @@
         <v>168.92</v>
       </c>
       <c r="F17" t="n">
+        <v>15.22</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1457.87</v>
+      </c>
+      <c r="H17" t="n">
         <v>22.51</v>
+      </c>
+      <c r="I17" t="n">
+        <v>7.04</v>
       </c>
     </row>
     <row r="18">
@@ -2054,6 +2111,15 @@
         <v>65.79000000000001</v>
       </c>
       <c r="F18" t="n">
+        <v>13.62</v>
+      </c>
+      <c r="G18" t="n">
+        <v>117.97</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="I18" t="n">
         <v>2.74</v>
       </c>
     </row>
@@ -2078,6 +2144,15 @@
         <v>134.32</v>
       </c>
       <c r="F19" t="n">
+        <v>134.32</v>
+      </c>
+      <c r="G19" t="n">
+        <v>134.32</v>
+      </c>
+      <c r="H19" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="I19" t="n">
         <v>5.6</v>
       </c>
     </row>
@@ -2102,7 +2177,16 @@
         <v>8.77</v>
       </c>
       <c r="F20" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G20" t="n">
+        <v>304.37</v>
+      </c>
+      <c r="H20" t="n">
         <v>2.47</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.37</v>
       </c>
     </row>
     <row r="21">
@@ -2126,7 +2210,16 @@
         <v>603.25</v>
       </c>
       <c r="F21" t="n">
+        <v>539.1799999999999</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1917.93</v>
+      </c>
+      <c r="H21" t="n">
         <v>42.5</v>
+      </c>
+      <c r="I21" t="n">
+        <v>25.14</v>
       </c>
     </row>
     <row r="22">
@@ -2150,7 +2243,16 @@
         <v>598.02</v>
       </c>
       <c r="F22" t="n">
+        <v>120.9</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2019.82</v>
+      </c>
+      <c r="H22" t="n">
         <v>31.32</v>
+      </c>
+      <c r="I22" t="n">
+        <v>24.92</v>
       </c>
     </row>
     <row r="23">
@@ -2174,7 +2276,16 @@
         <v>131.2</v>
       </c>
       <c r="F23" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G23" t="n">
+        <v>282.78</v>
+      </c>
+      <c r="H23" t="n">
         <v>5.76</v>
+      </c>
+      <c r="I23" t="n">
+        <v>5.47</v>
       </c>
     </row>
     <row r="24">
@@ -2198,7 +2309,16 @@
         <v>985.41</v>
       </c>
       <c r="F24" t="n">
+        <v>281.82</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1517.08</v>
+      </c>
+      <c r="H24" t="n">
         <v>39.27</v>
+      </c>
+      <c r="I24" t="n">
+        <v>41.06</v>
       </c>
     </row>
     <row r="25">
@@ -2222,7 +2342,16 @@
         <v>200.12</v>
       </c>
       <c r="F25" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1387.98</v>
+      </c>
+      <c r="H25" t="n">
         <v>13.53</v>
+      </c>
+      <c r="I25" t="n">
+        <v>8.34</v>
       </c>
     </row>
     <row r="26">
@@ -2246,7 +2375,16 @@
         <v>25.45</v>
       </c>
       <c r="F26" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="G26" t="n">
+        <v>356.45</v>
+      </c>
+      <c r="H26" t="n">
         <v>3.74</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1.06</v>
       </c>
     </row>
     <row r="27">
@@ -2270,6 +2408,15 @@
         <v>535.22</v>
       </c>
       <c r="F27" t="n">
+        <v>535.22</v>
+      </c>
+      <c r="G27" t="n">
+        <v>535.22</v>
+      </c>
+      <c r="H27" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="I27" t="n">
         <v>22.3</v>
       </c>
     </row>
@@ -2294,7 +2441,16 @@
         <v>143.28</v>
       </c>
       <c r="F28" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="G28" t="n">
+        <v>356.18</v>
+      </c>
+      <c r="H28" t="n">
         <v>6.84</v>
+      </c>
+      <c r="I28" t="n">
+        <v>5.97</v>
       </c>
     </row>
     <row r="29">
@@ -2318,6 +2474,15 @@
         <v>502.6</v>
       </c>
       <c r="F29" t="n">
+        <v>502.6</v>
+      </c>
+      <c r="G29" t="n">
+        <v>502.6</v>
+      </c>
+      <c r="H29" t="n">
+        <v>20.94</v>
+      </c>
+      <c r="I29" t="n">
         <v>20.94</v>
       </c>
     </row>
@@ -2342,7 +2507,16 @@
         <v>153.87</v>
       </c>
       <c r="F30" t="n">
+        <v>69.05</v>
+      </c>
+      <c r="G30" t="n">
+        <v>173.47</v>
+      </c>
+      <c r="H30" t="n">
         <v>6.18</v>
+      </c>
+      <c r="I30" t="n">
+        <v>6.41</v>
       </c>
     </row>
     <row r="31">
@@ -2366,6 +2540,15 @@
         <v>431.58</v>
       </c>
       <c r="F31" t="n">
+        <v>431.58</v>
+      </c>
+      <c r="G31" t="n">
+        <v>431.58</v>
+      </c>
+      <c r="H31" t="n">
+        <v>17.98</v>
+      </c>
+      <c r="I31" t="n">
         <v>17.98</v>
       </c>
     </row>
@@ -2390,7 +2573,16 @@
         <v>671.73</v>
       </c>
       <c r="F32" t="n">
+        <v>116</v>
+      </c>
+      <c r="G32" t="n">
+        <v>3716.62</v>
+      </c>
+      <c r="H32" t="n">
         <v>58.32</v>
+      </c>
+      <c r="I32" t="n">
+        <v>27.99</v>
       </c>
     </row>
     <row r="33">
@@ -2414,6 +2606,15 @@
         <v>409.54</v>
       </c>
       <c r="F33" t="n">
+        <v>164.65</v>
+      </c>
+      <c r="G33" t="n">
+        <v>654.4299999999999</v>
+      </c>
+      <c r="H33" t="n">
+        <v>17.06</v>
+      </c>
+      <c r="I33" t="n">
         <v>17.06</v>
       </c>
     </row>
@@ -2438,6 +2639,15 @@
         <v>115.56</v>
       </c>
       <c r="F34" t="n">
+        <v>66.81999999999999</v>
+      </c>
+      <c r="G34" t="n">
+        <v>164.3</v>
+      </c>
+      <c r="H34" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="I34" t="n">
         <v>4.82</v>
       </c>
     </row>
@@ -2462,7 +2672,16 @@
         <v>25.89</v>
       </c>
       <c r="F35" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="G35" t="n">
+        <v>541.97</v>
+      </c>
+      <c r="H35" t="n">
         <v>6.68</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1.08</v>
       </c>
     </row>
     <row r="36">
@@ -2486,7 +2705,16 @@
         <v>23.4</v>
       </c>
       <c r="F36" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1234.32</v>
+      </c>
+      <c r="H36" t="n">
         <v>5.55</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.98</v>
       </c>
     </row>
     <row r="37">
@@ -2510,31 +2738,49 @@
         <v>17.03</v>
       </c>
       <c r="F37" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G37" t="n">
+        <v>145.72</v>
+      </c>
+      <c r="H37" t="n">
         <v>1.51</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.71</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Request to deactivate template</t>
+          <t>Role or Group Assignment</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>WORKON 1.0</t>
+          <t>WORK ON NEXT GEN</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D38" t="n">
-        <v>862.87</v>
+        <v>111.42</v>
       </c>
       <c r="E38" t="n">
-        <v>862.87</v>
+        <v>3.08</v>
       </c>
       <c r="F38" t="n">
-        <v>35.95</v>
+        <v>0.18</v>
+      </c>
+      <c r="G38" t="n">
+        <v>538.92</v>
+      </c>
+      <c r="H38" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.13</v>
       </c>
     </row>
     <row r="39">
@@ -2545,44 +2791,62 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>WORK ON NEXT GEN</t>
+          <t>WORKON 1.0</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>9</v>
+        <v>76</v>
       </c>
       <c r="D39" t="n">
-        <v>111.42</v>
+        <v>261.05</v>
       </c>
       <c r="E39" t="n">
-        <v>3.08</v>
+        <v>38.38</v>
       </c>
       <c r="F39" t="n">
-        <v>4.64</v>
+        <v>0.4</v>
+      </c>
+      <c r="G39" t="n">
+        <v>3747.8</v>
+      </c>
+      <c r="H39" t="n">
+        <v>10.88</v>
+      </c>
+      <c r="I39" t="n">
+        <v>1.6</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Role or Group Assignment</t>
+          <t>SUBSTITUTE</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>WORKON 1.0</t>
+          <t>WORK ON NEXT GEN</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>76</v>
+        <v>27</v>
       </c>
       <c r="D40" t="n">
-        <v>261.05</v>
+        <v>205.33</v>
       </c>
       <c r="E40" t="n">
-        <v>38.38</v>
+        <v>32.65</v>
       </c>
       <c r="F40" t="n">
-        <v>10.88</v>
+        <v>0.08</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1224.93</v>
+      </c>
+      <c r="H40" t="n">
+        <v>8.56</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1.36</v>
       </c>
     </row>
     <row r="41">
@@ -2593,26 +2857,35 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>WORK ON NEXT GEN</t>
+          <t>WORKON 1.0</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>27</v>
+        <v>132</v>
       </c>
       <c r="D41" t="n">
-        <v>205.33</v>
+        <v>157.57</v>
       </c>
       <c r="E41" t="n">
-        <v>32.65</v>
+        <v>73.25</v>
       </c>
       <c r="F41" t="n">
-        <v>8.56</v>
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G41" t="n">
+        <v>985.95</v>
+      </c>
+      <c r="H41" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="I41" t="n">
+        <v>3.05</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SUBSTITUTE</t>
+          <t>Server issue</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2621,40 +2894,58 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>132</v>
+        <v>327</v>
       </c>
       <c r="D42" t="n">
-        <v>157.57</v>
+        <v>762.37</v>
       </c>
       <c r="E42" t="n">
-        <v>73.25</v>
+        <v>530.13</v>
       </c>
       <c r="F42" t="n">
-        <v>6.57</v>
+        <v>2.32</v>
+      </c>
+      <c r="G42" t="n">
+        <v>3089.68</v>
+      </c>
+      <c r="H42" t="n">
+        <v>31.77</v>
+      </c>
+      <c r="I42" t="n">
+        <v>22.09</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Server issue</t>
+          <t>Synchronize User Information</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>WORKON 1.0</t>
+          <t>WORK ON NEXT GEN</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>327</v>
+        <v>2</v>
       </c>
       <c r="D43" t="n">
-        <v>762.37</v>
+        <v>176.47</v>
       </c>
       <c r="E43" t="n">
-        <v>530.13</v>
+        <v>176.47</v>
       </c>
       <c r="F43" t="n">
-        <v>31.77</v>
+        <v>67.58</v>
+      </c>
+      <c r="G43" t="n">
+        <v>285.35</v>
+      </c>
+      <c r="H43" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="I43" t="n">
+        <v>7.35</v>
       </c>
     </row>
     <row r="44">
@@ -2665,122 +2956,167 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>WORK ON NEXT GEN</t>
+          <t>WORKON 1.0</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D44" t="n">
-        <v>176.47</v>
+        <v>117.46</v>
       </c>
       <c r="E44" t="n">
-        <v>176.47</v>
+        <v>46.14</v>
       </c>
       <c r="F44" t="n">
-        <v>7.35</v>
+        <v>0.97</v>
+      </c>
+      <c r="G44" t="n">
+        <v>479.92</v>
+      </c>
+      <c r="H44" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1.92</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Synchronize User Information</t>
+          <t>UIB issue</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>WORKON 1.0</t>
+          <t>WORK ON NEXT GEN</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D45" t="n">
-        <v>117.46</v>
+        <v>349.86</v>
       </c>
       <c r="E45" t="n">
-        <v>46.14</v>
+        <v>406.28</v>
       </c>
       <c r="F45" t="n">
-        <v>4.89</v>
+        <v>1.28</v>
+      </c>
+      <c r="G45" t="n">
+        <v>679.05</v>
+      </c>
+      <c r="H45" t="n">
+        <v>14.58</v>
+      </c>
+      <c r="I45" t="n">
+        <v>16.93</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Timeline for new feature</t>
+          <t>UIB issue</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>WORK ON NEXT GEN</t>
+          <t>WORKON 1.0</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D46" t="n">
-        <v>1204.42</v>
+        <v>338.31</v>
       </c>
       <c r="E46" t="n">
-        <v>1204.42</v>
+        <v>350.22</v>
       </c>
       <c r="F46" t="n">
-        <v>50.18</v>
+        <v>24.85</v>
+      </c>
+      <c r="G46" t="n">
+        <v>627.95</v>
+      </c>
+      <c r="H46" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="I46" t="n">
+        <v>14.59</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>UIB issue</t>
+          <t>UNCLASSIFIED</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>WORK ON NEXT GEN</t>
+          <t>WORKON 1.0</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>349.86</v>
+        <v>184.77</v>
       </c>
       <c r="E47" t="n">
-        <v>406.28</v>
+        <v>184.77</v>
       </c>
       <c r="F47" t="n">
-        <v>14.58</v>
+        <v>184.77</v>
+      </c>
+      <c r="G47" t="n">
+        <v>184.77</v>
+      </c>
+      <c r="H47" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="I47" t="n">
+        <v>7.7</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>UIB issue</t>
+          <t>Update approver</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>WORKON 1.0</t>
+          <t>WORK ON NEXT GEN</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D48" t="n">
-        <v>338.31</v>
+        <v>437.17</v>
       </c>
       <c r="E48" t="n">
-        <v>350.22</v>
+        <v>437.17</v>
       </c>
       <c r="F48" t="n">
-        <v>14.1</v>
+        <v>437.17</v>
+      </c>
+      <c r="G48" t="n">
+        <v>437.17</v>
+      </c>
+      <c r="H48" t="n">
+        <v>18.22</v>
+      </c>
+      <c r="I48" t="n">
+        <v>18.22</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>UNCLASSIFIED</t>
+          <t>Update approver</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2789,22 +3125,31 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="D49" t="n">
-        <v>184.77</v>
+        <v>187.47</v>
       </c>
       <c r="E49" t="n">
-        <v>184.77</v>
+        <v>96.23</v>
       </c>
       <c r="F49" t="n">
-        <v>7.7</v>
+        <v>2.23</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1275.23</v>
+      </c>
+      <c r="H49" t="n">
+        <v>7.81</v>
+      </c>
+      <c r="I49" t="n">
+        <v>4.01</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Update approver</t>
+          <t>Update data in form</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2813,22 +3158,31 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D50" t="n">
-        <v>437.17</v>
+        <v>514.59</v>
       </c>
       <c r="E50" t="n">
-        <v>437.17</v>
+        <v>514.59</v>
       </c>
       <c r="F50" t="n">
-        <v>18.22</v>
+        <v>500.97</v>
+      </c>
+      <c r="G50" t="n">
+        <v>528.22</v>
+      </c>
+      <c r="H50" t="n">
+        <v>21.44</v>
+      </c>
+      <c r="I50" t="n">
+        <v>21.44</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Update approver</t>
+          <t>Update data in form</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2837,22 +3191,31 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D51" t="n">
-        <v>187.47</v>
+        <v>95.55</v>
       </c>
       <c r="E51" t="n">
-        <v>96.23</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="F51" t="n">
-        <v>7.81</v>
+        <v>0.68</v>
+      </c>
+      <c r="G51" t="n">
+        <v>245.85</v>
+      </c>
+      <c r="H51" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="I51" t="n">
+        <v>3.89</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Update data in form</t>
+          <t>Update redirection configuration</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2861,22 +3224,31 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>514.59</v>
+        <v>24.85</v>
       </c>
       <c r="E52" t="n">
-        <v>514.59</v>
+        <v>24.85</v>
       </c>
       <c r="F52" t="n">
-        <v>21.44</v>
+        <v>24.85</v>
+      </c>
+      <c r="G52" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="H52" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="I52" t="n">
+        <v>1.04</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Update data in form</t>
+          <t>Update redirection configuration</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2885,63 +3257,24 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>95.55</v>
+        <v>100.73</v>
       </c>
       <c r="E53" t="n">
-        <v>93.40000000000001</v>
+        <v>100.73</v>
       </c>
       <c r="F53" t="n">
-        <v>3.98</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Update redirection configuration</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>WORK ON NEXT GEN</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>1</v>
-      </c>
-      <c r="D54" t="n">
-        <v>24.85</v>
-      </c>
-      <c r="E54" t="n">
-        <v>24.85</v>
-      </c>
-      <c r="F54" t="n">
-        <v>1.04</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Update redirection configuration</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>WORKON 1.0</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" t="n">
         <v>100.73</v>
       </c>
-      <c r="E55" t="n">
+      <c r="G53" t="n">
         <v>100.73</v>
       </c>
-      <c r="F55" t="n">
+      <c r="H53" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="I53" t="n">
         <v>4.2</v>
       </c>
     </row>
@@ -2956,21 +3289,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Count</t>
@@ -2983,91 +3310,84 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Median_Hours</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Min_Hours</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Max_Hours</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Avg_Days</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Median_Hours</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Median_Days</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Min_Hours</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Max_Hours</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Service</t>
-        </is>
+          <t>WORK ON NEXT GEN</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>176</v>
+      </c>
+      <c r="C2" t="n">
+        <v>255.65</v>
+      </c>
+      <c r="D2" t="n">
+        <v>119.49</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1960.83</v>
+      </c>
+      <c r="G2" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4.98</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WORK ON NEXT GEN</t>
+          <t>WORKON 1.0</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>176</v>
+        <v>1440</v>
       </c>
       <c r="C3" t="n">
-        <v>255.65</v>
+        <v>361.43</v>
       </c>
       <c r="D3" t="n">
-        <v>10.65</v>
+        <v>165.11</v>
       </c>
       <c r="E3" t="n">
-        <v>119.49</v>
+        <v>0.05</v>
       </c>
       <c r="F3" t="n">
-        <v>4.98</v>
+        <v>3747.8</v>
       </c>
       <c r="G3" t="n">
-        <v>0.08</v>
+        <v>15.06</v>
       </c>
       <c r="H3" t="n">
-        <v>1960.83</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>WORKON 1.0</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1440</v>
-      </c>
-      <c r="C4" t="n">
-        <v>361.43</v>
-      </c>
-      <c r="D4" t="n">
-        <v>15.06</v>
-      </c>
-      <c r="E4" t="n">
-        <v>165.11</v>
-      </c>
-      <c r="F4" t="n">
         <v>6.88</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H4" t="n">
-        <v>3747.8</v>
       </c>
     </row>
   </sheetData>
@@ -3081,172 +3401,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>📊 OVERALL METRICS</t>
-        </is>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Total Tickets</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>1616</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Total Tickets</t>
+          <t>Total Groupings</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1616</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Total Groupings</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Avg Resolution Time (days)</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>14.58</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Median Resolution Time (days)</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>6.48</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>⚡ TOP 5 FASTEST ISSUES</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Request account for user</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1.51</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Access issue (with workon templates)</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>2.26</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Create issue workon template</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>2.47</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Update redirection configuration</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>2.62</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Chatbot issue</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>3.69</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>🐌 TOP 5 SLOWEST ISSUES</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Notification Failures</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>51.59</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Timeline for new feature</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>50.18</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Request to deactivate template</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>35.95</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Create new app</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>35.05</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Server issue</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>31.77</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>